<commit_message>
campo magnetico de la tierra
</commit_message>
<xml_diff>
--- a/Electromagnetismo/practica5magnetierra/p5electro.xlsx
+++ b/Electromagnetismo/practica5magnetierra/p5electro.xlsx
@@ -5,18 +5,20 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alex\Plotting\Electromagnetismo\practica5magnetierra\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alex\Proyectos\PythonPlotting\Electromagnetismo\practica5magnetierra\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A6F78076-3F0E-42CB-8AF4-2D912B4E18AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2F9E8088-BC46-4F72-9E08-E04BB69C537C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{5784CD7F-D9FE-48D9-9F16-4B8A459F24D7}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{5784CD7F-D9FE-48D9-9F16-4B8A459F24D7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
     <sheet name="Sheet4" sheetId="4" r:id="rId4"/>
+    <sheet name="Sheet5" sheetId="5" r:id="rId5"/>
+    <sheet name="Sheet6" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="4">
   <si>
     <t>I (A)</t>
   </si>
@@ -61,9 +63,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="#,##0.000"/>
+    <numFmt numFmtId="164" formatCode="#,##0.000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -84,7 +86,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -127,6 +129,12 @@
         <bgColor rgb="FFFCE5CD"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -156,7 +164,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -164,7 +172,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -176,37 +184,22 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -545,9 +538,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7DD8CE0-63AB-4230-AADF-A44B57D6D9BB}">
   <dimension ref="A1:D16"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" ht="15.75" thickTop="1" thickBot="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -561,214 +554,214 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" ht="15.75" thickTop="1" thickBot="1">
       <c r="A2" s="1">
         <v>-0.221</v>
       </c>
       <c r="B2" s="2">
-        <v>7.9000000000000001E-4</v>
+        <v>5.2100000000000002E-3</v>
       </c>
       <c r="C2" s="1">
         <v>80</v>
       </c>
       <c r="D2" s="2">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+        <v>0.28867513500000003</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="15.75" thickTop="1" thickBot="1">
       <c r="A3" s="1">
         <v>-0.14199999999999999</v>
       </c>
       <c r="B3" s="2">
-        <v>1.58E-3</v>
+        <v>4.4200000000000003E-3</v>
       </c>
       <c r="C3" s="1">
         <v>74</v>
       </c>
       <c r="D3" s="2">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+        <v>0.28867513500000003</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="15.75" thickTop="1" thickBot="1">
       <c r="A4" s="1">
         <v>-0.104</v>
       </c>
       <c r="B4" s="2">
-        <v>1.9599999999999999E-3</v>
+        <v>4.0400000000000002E-3</v>
       </c>
       <c r="C4" s="1">
         <v>70</v>
       </c>
       <c r="D4" s="2">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+        <v>0.28867513500000003</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="15.75" thickTop="1" thickBot="1">
       <c r="A5" s="1">
         <v>-7.4999999999999997E-2</v>
       </c>
       <c r="B5" s="2">
-        <v>2.2499999999999998E-3</v>
+        <v>3.7499999999999999E-3</v>
       </c>
       <c r="C5" s="1">
         <v>64</v>
       </c>
       <c r="D5" s="2">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+        <v>0.28867513500000003</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="15.75" thickTop="1" thickBot="1">
       <c r="A6" s="3">
         <v>-6.4000000000000001E-2</v>
       </c>
       <c r="B6" s="2">
-        <v>2.3600000000000001E-3</v>
+        <v>3.64E-3</v>
       </c>
       <c r="C6" s="1">
         <v>60</v>
       </c>
       <c r="D6" s="2">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+        <v>0.28867513500000003</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="15.75" thickTop="1" thickBot="1">
       <c r="A7" s="1">
         <v>-4.9000000000000002E-2</v>
       </c>
       <c r="B7" s="2">
-        <v>2.5100000000000001E-3</v>
+        <v>3.49E-3</v>
       </c>
       <c r="C7" s="1">
         <v>54</v>
       </c>
       <c r="D7" s="2">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+        <v>0.28867513500000003</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="15.75" thickTop="1" thickBot="1">
       <c r="A8" s="1">
         <v>-4.4999999999999998E-2</v>
       </c>
       <c r="B8" s="2">
-        <v>2.5500000000000002E-3</v>
+        <v>3.4499999999999999E-3</v>
       </c>
       <c r="C8" s="1">
         <v>50</v>
       </c>
       <c r="D8" s="2">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+        <v>0.28867513500000003</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="15.75" thickTop="1" thickBot="1">
       <c r="A9" s="1">
         <v>-3.3000000000000002E-2</v>
       </c>
       <c r="B9" s="2">
-        <v>2.6700000000000001E-3</v>
+        <v>3.3300000000000001E-3</v>
       </c>
       <c r="C9" s="1">
         <v>44</v>
       </c>
       <c r="D9" s="2">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+        <v>0.28867513500000003</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="15.75" thickTop="1" thickBot="1">
       <c r="A10" s="1">
         <v>-2.9000000000000001E-2</v>
       </c>
       <c r="B10" s="2">
-        <v>2.7100000000000002E-3</v>
+        <v>3.29E-3</v>
       </c>
       <c r="C10" s="1">
         <v>40</v>
       </c>
       <c r="D10" s="2">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+        <v>0.28867513500000003</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="15.75" thickTop="1" thickBot="1">
       <c r="A11" s="1">
         <v>-2.1999999999999999E-2</v>
       </c>
       <c r="B11" s="2">
-        <v>2.7799999999999999E-3</v>
+        <v>3.2200000000000002E-3</v>
       </c>
       <c r="C11" s="1">
         <v>34</v>
       </c>
       <c r="D11" s="2">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+        <v>0.28867513500000003</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="15.75" thickTop="1" thickBot="1">
       <c r="A12" s="1">
         <v>-1.9E-2</v>
       </c>
       <c r="B12" s="2">
-        <v>2.81E-3</v>
+        <v>3.1900000000000001E-3</v>
       </c>
       <c r="C12" s="1">
         <v>30</v>
       </c>
       <c r="D12" s="2">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+        <v>0.28867513500000003</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="15.75" thickTop="1" thickBot="1">
       <c r="A13" s="4">
         <v>-1.4999999999999999E-2</v>
       </c>
       <c r="B13" s="4">
-        <v>2.8500000000000001E-3</v>
+        <v>3.15E-3</v>
       </c>
       <c r="C13" s="4">
         <v>24</v>
       </c>
       <c r="D13" s="4">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+        <v>0.28867513500000003</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="15.75" thickTop="1" thickBot="1">
       <c r="A14" s="5">
         <v>-1.2E-2</v>
       </c>
       <c r="B14" s="5">
-        <v>2.8800000000000002E-3</v>
+        <v>3.1199999999999999E-3</v>
       </c>
       <c r="C14" s="5">
         <v>20</v>
       </c>
       <c r="D14" s="5">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+        <v>0.28867513500000003</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="15.75" thickTop="1" thickBot="1">
       <c r="A15" s="5">
         <v>-8.0000000000000002E-3</v>
       </c>
       <c r="B15" s="5">
-        <v>2.9199999999999999E-3</v>
+        <v>3.0799999999999998E-3</v>
       </c>
       <c r="C15" s="5">
         <v>14</v>
       </c>
       <c r="D15" s="5">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+        <v>0.28867513500000003</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="15.75" thickTop="1" thickBot="1">
       <c r="A16" s="6">
         <v>-6.0000000000000001E-3</v>
       </c>
       <c r="B16" s="6">
-        <v>2.9399999999999999E-3</v>
+        <v>3.0599999999999998E-3</v>
       </c>
       <c r="C16" s="6">
         <v>10</v>
       </c>
       <c r="D16" s="6">
-        <v>0.28867513459999999</v>
+        <v>0.28867513500000003</v>
       </c>
     </row>
   </sheetData>
@@ -779,9 +772,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE547059-393E-4D64-BA7C-1947BE889733}">
   <dimension ref="A1:D16"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -795,214 +788,244 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
       <c r="A2" s="7">
         <v>0.19400000000000001</v>
       </c>
       <c r="B2" s="8">
+        <f t="shared" ref="B2:B16" si="0">ABS(A2*(1/100))+0.003</f>
         <v>4.9399999999999999E-3</v>
       </c>
       <c r="C2" s="7">
         <v>80</v>
       </c>
       <c r="D2" s="8">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" ref="D2:D16" si="1">1/SQRT(12)</f>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
       <c r="A3" s="7">
         <v>0.13100000000000001</v>
       </c>
       <c r="B3" s="8">
-        <v>4.3099999999999996E-3</v>
+        <f t="shared" si="0"/>
+        <v>4.3100000000000005E-3</v>
       </c>
       <c r="C3" s="7">
         <v>74</v>
       </c>
       <c r="D3" s="8">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
       <c r="A4" s="7">
         <v>0.104</v>
       </c>
       <c r="B4" s="8">
+        <f t="shared" si="0"/>
         <v>4.0400000000000002E-3</v>
       </c>
       <c r="C4" s="7">
         <v>70</v>
       </c>
       <c r="D4" s="8">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
       <c r="A5" s="7">
         <v>7.9000000000000001E-2</v>
       </c>
       <c r="B5" s="8">
+        <f t="shared" si="0"/>
         <v>3.79E-3</v>
       </c>
       <c r="C5" s="7">
         <v>64</v>
       </c>
       <c r="D5" s="8">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
       <c r="A6" s="9">
         <v>6.8000000000000005E-2</v>
       </c>
       <c r="B6" s="8">
+        <f t="shared" si="0"/>
         <v>3.6800000000000001E-3</v>
       </c>
       <c r="C6" s="7">
         <v>60</v>
       </c>
       <c r="D6" s="8">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
       <c r="A7" s="7">
         <v>5.2999999999999999E-2</v>
       </c>
       <c r="B7" s="8">
+        <f t="shared" si="0"/>
         <v>3.5300000000000002E-3</v>
       </c>
       <c r="C7" s="7">
         <v>54</v>
       </c>
       <c r="D7" s="8">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
       <c r="A8" s="7">
         <v>4.7E-2</v>
       </c>
       <c r="B8" s="8">
+        <f t="shared" si="0"/>
         <v>3.47E-3</v>
       </c>
       <c r="C8" s="7">
         <v>50</v>
       </c>
       <c r="D8" s="8">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
       <c r="A9" s="7">
         <v>3.6999999999999998E-2</v>
       </c>
       <c r="B9" s="8">
+        <f t="shared" si="0"/>
         <v>3.3700000000000002E-3</v>
       </c>
       <c r="C9" s="7">
         <v>44</v>
       </c>
       <c r="D9" s="8">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
       <c r="A10" s="7">
         <v>3.3000000000000002E-2</v>
       </c>
       <c r="B10" s="8">
+        <f t="shared" si="0"/>
         <v>3.3300000000000001E-3</v>
       </c>
       <c r="C10" s="7">
         <v>40</v>
       </c>
       <c r="D10" s="8">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
       <c r="A11" s="7">
         <v>2.8000000000000001E-2</v>
       </c>
       <c r="B11" s="8">
+        <f t="shared" si="0"/>
         <v>3.2799999999999999E-3</v>
       </c>
       <c r="C11" s="7">
         <v>34</v>
       </c>
       <c r="D11" s="8">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
       <c r="A12" s="7">
         <v>2.4E-2</v>
       </c>
       <c r="B12" s="8">
-        <v>3.2399999999999998E-3</v>
+        <f t="shared" si="0"/>
+        <v>3.2400000000000003E-3</v>
       </c>
       <c r="C12" s="7">
         <v>30</v>
       </c>
       <c r="D12" s="8">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
       <c r="A13" s="7">
         <v>1.9E-2</v>
       </c>
       <c r="B13" s="8">
+        <f t="shared" si="0"/>
         <v>3.1900000000000001E-3</v>
       </c>
       <c r="C13" s="7">
         <v>24</v>
       </c>
       <c r="D13" s="8">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
       <c r="A14" s="7">
         <v>1.6E-2</v>
       </c>
       <c r="B14" s="8">
+        <f t="shared" si="0"/>
         <v>3.16E-3</v>
       </c>
       <c r="C14" s="7">
         <v>20</v>
       </c>
       <c r="D14" s="8">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
       <c r="A15" s="7">
         <v>1.0999999999999999E-2</v>
       </c>
       <c r="B15" s="8">
+        <f t="shared" si="0"/>
         <v>3.1099999999999999E-3</v>
       </c>
       <c r="C15" s="7">
         <v>14</v>
       </c>
       <c r="D15" s="8">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
       <c r="A16" s="7">
         <v>8.0000000000000002E-3</v>
       </c>
       <c r="B16" s="8">
-        <v>3.0799999999999998E-3</v>
+        <f t="shared" si="0"/>
+        <v>3.0800000000000003E-3</v>
       </c>
       <c r="C16" s="7">
         <v>10</v>
       </c>
       <c r="D16" s="8">
-        <v>0.28867513459999999</v>
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
       </c>
     </row>
   </sheetData>
@@ -1013,230 +1036,260 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2F4E541-1C32-4366-9AC7-36ECD3FB3D26}">
   <dimension ref="A1:D16"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="8" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="10">
+    <row r="2" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A2" s="7">
         <v>-0.25900000000000001</v>
       </c>
-      <c r="B2" s="11">
-        <v>4.0999999999999999E-4</v>
-      </c>
-      <c r="C2" s="10">
+      <c r="B2" s="8">
+        <f t="shared" ref="B2:B16" si="0">ABS(A2*(1/100))+0.003</f>
+        <v>5.5900000000000004E-3</v>
+      </c>
+      <c r="C2" s="7">
         <v>80</v>
       </c>
-      <c r="D2" s="11">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="10">
+      <c r="D2" s="8">
+        <f t="shared" ref="D2:D16" si="1">1/SQRT(12)</f>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A3" s="7">
         <v>-0.156</v>
       </c>
-      <c r="B3" s="11">
-        <v>1.4400000000000001E-3</v>
-      </c>
-      <c r="C3" s="10">
+      <c r="B3" s="8">
+        <f t="shared" si="0"/>
+        <v>4.5599999999999998E-3</v>
+      </c>
+      <c r="C3" s="7">
         <v>74</v>
       </c>
-      <c r="D3" s="11">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="10">
+      <c r="D3" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A4" s="7">
         <v>-0.109</v>
       </c>
-      <c r="B4" s="11">
-        <v>1.91E-3</v>
-      </c>
-      <c r="C4" s="10">
+      <c r="B4" s="8">
+        <f t="shared" si="0"/>
+        <v>4.0899999999999999E-3</v>
+      </c>
+      <c r="C4" s="7">
         <v>70</v>
       </c>
-      <c r="D4" s="11">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="10">
+      <c r="D4" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A5" s="7">
         <v>-8.7999999999999995E-2</v>
       </c>
-      <c r="B5" s="11">
-        <v>2.1199999999999999E-3</v>
-      </c>
-      <c r="C5" s="10">
+      <c r="B5" s="8">
+        <f t="shared" si="0"/>
+        <v>3.8799999999999998E-3</v>
+      </c>
+      <c r="C5" s="7">
         <v>64</v>
       </c>
-      <c r="D5" s="11">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="12">
+      <c r="D5" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A6" s="9">
         <v>-7.2999999999999995E-2</v>
       </c>
-      <c r="B6" s="11">
-        <v>2.2699999999999999E-3</v>
-      </c>
-      <c r="C6" s="10">
+      <c r="B6" s="8">
+        <f t="shared" si="0"/>
+        <v>3.7299999999999998E-3</v>
+      </c>
+      <c r="C6" s="7">
         <v>60</v>
       </c>
-      <c r="D6" s="11">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="10">
+      <c r="D6" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A7" s="7">
         <v>-5.7000000000000002E-2</v>
       </c>
-      <c r="B7" s="11">
-        <v>2.4299999999999999E-3</v>
-      </c>
-      <c r="C7" s="10">
+      <c r="B7" s="8">
+        <f t="shared" si="0"/>
+        <v>3.5700000000000003E-3</v>
+      </c>
+      <c r="C7" s="7">
         <v>54</v>
       </c>
-      <c r="D7" s="11">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="10">
+      <c r="D7" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A8" s="7">
         <v>-4.8000000000000001E-2</v>
       </c>
-      <c r="B8" s="11">
-        <v>2.5200000000000001E-3</v>
-      </c>
-      <c r="C8" s="10">
+      <c r="B8" s="8">
+        <f t="shared" si="0"/>
+        <v>3.48E-3</v>
+      </c>
+      <c r="C8" s="7">
         <v>50</v>
       </c>
-      <c r="D8" s="11">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="10">
+      <c r="D8" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A9" s="7">
         <v>-0.04</v>
       </c>
-      <c r="B9" s="11">
-        <v>2.5999999999999999E-3</v>
-      </c>
-      <c r="C9" s="10">
+      <c r="B9" s="8">
+        <f t="shared" si="0"/>
+        <v>3.4000000000000002E-3</v>
+      </c>
+      <c r="C9" s="7">
         <v>44</v>
       </c>
-      <c r="D9" s="11">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="10">
+      <c r="D9" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A10" s="7">
         <v>-3.5000000000000003E-2</v>
       </c>
-      <c r="B10" s="11">
-        <v>2.65E-3</v>
-      </c>
-      <c r="C10" s="10">
+      <c r="B10" s="8">
+        <f t="shared" si="0"/>
+        <v>3.3500000000000001E-3</v>
+      </c>
+      <c r="C10" s="7">
         <v>40</v>
       </c>
-      <c r="D10" s="11">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="10">
+      <c r="D10" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A11" s="7">
         <v>-2.7E-2</v>
       </c>
-      <c r="B11" s="11">
-        <v>2.7299999999999998E-3</v>
-      </c>
-      <c r="C11" s="10">
+      <c r="B11" s="8">
+        <f t="shared" si="0"/>
+        <v>3.2699999999999999E-3</v>
+      </c>
+      <c r="C11" s="7">
         <v>34</v>
       </c>
-      <c r="D11" s="11">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="10">
+      <c r="D11" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A12" s="7">
         <v>-2.3E-2</v>
       </c>
-      <c r="B12" s="11">
-        <v>2.7699999999999999E-3</v>
-      </c>
-      <c r="C12" s="10">
+      <c r="B12" s="8">
+        <f t="shared" si="0"/>
+        <v>3.2300000000000002E-3</v>
+      </c>
+      <c r="C12" s="7">
         <v>30</v>
       </c>
-      <c r="D12" s="11">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="10">
+      <c r="D12" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A13" s="7">
         <v>-1.7000000000000001E-2</v>
       </c>
-      <c r="B13" s="11">
-        <v>2.8300000000000001E-3</v>
-      </c>
-      <c r="C13" s="10">
+      <c r="B13" s="8">
+        <f t="shared" si="0"/>
+        <v>3.1700000000000001E-3</v>
+      </c>
+      <c r="C13" s="7">
         <v>24</v>
       </c>
-      <c r="D13" s="11">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="10">
+      <c r="D13" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A14" s="7">
         <v>-1.2999999999999999E-2</v>
       </c>
-      <c r="B14" s="11">
-        <v>2.8700000000000002E-3</v>
-      </c>
-      <c r="C14" s="10">
+      <c r="B14" s="8">
+        <f t="shared" si="0"/>
+        <v>3.13E-3</v>
+      </c>
+      <c r="C14" s="7">
         <v>20</v>
       </c>
-      <c r="D14" s="11">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="10">
+      <c r="D14" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A15" s="7">
         <v>-0.01</v>
       </c>
-      <c r="B15" s="11">
-        <v>2.8999999999999998E-3</v>
-      </c>
-      <c r="C15" s="10">
+      <c r="B15" s="8">
+        <f t="shared" si="0"/>
+        <v>3.0999999999999999E-3</v>
+      </c>
+      <c r="C15" s="7">
         <v>14</v>
       </c>
-      <c r="D15" s="11">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="10">
+      <c r="D15" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A16" s="7">
         <v>-7.0000000000000001E-3</v>
       </c>
-      <c r="B16" s="11">
-        <v>2.9299999999999999E-3</v>
-      </c>
-      <c r="C16" s="10">
+      <c r="B16" s="8">
+        <f t="shared" si="0"/>
+        <v>3.0700000000000002E-3</v>
+      </c>
+      <c r="C16" s="7">
         <v>10</v>
       </c>
-      <c r="D16" s="11">
-        <v>0.28867513459999999</v>
+      <c r="D16" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
       </c>
     </row>
   </sheetData>
@@ -1247,232 +1300,792 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3B254D7-07D4-4BFC-A32C-1EEC6A576A5C}">
   <dimension ref="A1:D16"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="13" t="s">
+    <row r="1" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="8" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="13">
+    <row r="2" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A2" s="7">
         <v>0.19</v>
       </c>
-      <c r="B2" s="14">
+      <c r="B2" s="8">
+        <f t="shared" ref="B2:B16" si="0">ABS(A2*(1/100))+0.003</f>
         <v>4.8999999999999998E-3</v>
       </c>
-      <c r="C2" s="13">
+      <c r="C2" s="7">
         <v>80</v>
       </c>
-      <c r="D2" s="14">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="13">
+      <c r="D2" s="8">
+        <f t="shared" ref="D2:D16" si="1">1/SQRT(12)</f>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A3" s="7">
         <v>0.122</v>
       </c>
-      <c r="B3" s="14">
+      <c r="B3" s="8">
+        <f t="shared" si="0"/>
         <v>4.2199999999999998E-3</v>
       </c>
-      <c r="C3" s="13">
+      <c r="C3" s="7">
         <v>74</v>
       </c>
-      <c r="D3" s="14">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="13">
+      <c r="D3" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A4" s="7">
         <v>0.10299999999999999</v>
       </c>
-      <c r="B4" s="14">
+      <c r="B4" s="8">
+        <f t="shared" si="0"/>
         <v>4.0299999999999997E-3</v>
       </c>
-      <c r="C4" s="13">
+      <c r="C4" s="7">
         <v>70</v>
       </c>
-      <c r="D4" s="14">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="16">
+      <c r="D4" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A5" s="10">
         <v>7.9000000000000001E-2</v>
       </c>
-      <c r="B5" s="14">
+      <c r="B5" s="8">
+        <f t="shared" si="0"/>
         <v>3.79E-3</v>
       </c>
-      <c r="C5" s="13">
+      <c r="C5" s="7">
         <v>64</v>
       </c>
-      <c r="D5" s="14">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="15">
+      <c r="D5" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A6" s="9">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="B6" s="14">
+      <c r="B6" s="8">
+        <f t="shared" si="0"/>
         <v>3.65E-3</v>
       </c>
-      <c r="C6" s="13">
+      <c r="C6" s="7">
         <v>60</v>
       </c>
-      <c r="D6" s="14">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="17">
-        <v>0.06</v>
-      </c>
-      <c r="B7" s="17">
-        <v>3.5999999999999999E-3</v>
-      </c>
-      <c r="C7" s="17">
+      <c r="D6" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A7" s="11">
+        <v>5.6000000000000001E-2</v>
+      </c>
+      <c r="B7" s="8">
+        <f t="shared" si="0"/>
+        <v>3.5600000000000002E-3</v>
+      </c>
+      <c r="C7" s="11">
         <v>54</v>
       </c>
-      <c r="D7" s="17">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="13">
+      <c r="D7" s="11">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A8" s="7">
         <v>4.3999999999999997E-2</v>
       </c>
-      <c r="B8" s="14">
+      <c r="B8" s="8">
+        <f t="shared" si="0"/>
         <v>3.4399999999999999E-3</v>
       </c>
-      <c r="C8" s="13">
+      <c r="C8" s="7">
         <v>50</v>
       </c>
-      <c r="D8" s="14">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="13">
+      <c r="D8" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A9" s="7">
         <v>3.5999999999999997E-2</v>
       </c>
-      <c r="B9" s="14">
+      <c r="B9" s="8">
+        <f t="shared" si="0"/>
         <v>3.3600000000000001E-3</v>
       </c>
-      <c r="C9" s="13">
+      <c r="C9" s="7">
         <v>44</v>
       </c>
-      <c r="D9" s="14">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="13">
+      <c r="D9" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A10" s="7">
         <v>3.1E-2</v>
       </c>
-      <c r="B10" s="14">
+      <c r="B10" s="8">
+        <f t="shared" si="0"/>
         <v>3.31E-3</v>
       </c>
-      <c r="C10" s="13">
+      <c r="C10" s="7">
         <v>40</v>
       </c>
-      <c r="D10" s="14">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="13">
+      <c r="D10" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A11" s="7">
         <v>2.5999999999999999E-2</v>
       </c>
-      <c r="B11" s="14">
+      <c r="B11" s="8">
+        <f t="shared" si="0"/>
         <v>3.2599999999999999E-3</v>
       </c>
-      <c r="C11" s="13">
+      <c r="C11" s="7">
         <v>34</v>
       </c>
-      <c r="D11" s="14">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="13">
+      <c r="D11" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A12" s="7">
         <v>2.3E-2</v>
       </c>
-      <c r="B12" s="14">
-        <v>3.2299999999999998E-3</v>
-      </c>
-      <c r="C12" s="13">
+      <c r="B12" s="8">
+        <f t="shared" si="0"/>
+        <v>3.2300000000000002E-3</v>
+      </c>
+      <c r="C12" s="7">
         <v>30</v>
       </c>
-      <c r="D12" s="14">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="17">
-        <v>2.4E-2</v>
-      </c>
-      <c r="B13" s="17">
-        <v>3.2399999999999998E-3</v>
-      </c>
-      <c r="C13" s="17">
+      <c r="D12" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A13" s="11">
+        <v>1.6E-2</v>
+      </c>
+      <c r="B13" s="8">
+        <f t="shared" si="0"/>
+        <v>3.16E-3</v>
+      </c>
+      <c r="C13" s="11">
         <v>24</v>
       </c>
-      <c r="D13" s="17">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="17">
+      <c r="D13" s="11">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A14" s="12">
         <v>1.2999999999999999E-2</v>
       </c>
-      <c r="B14" s="17">
+      <c r="B14" s="8">
+        <f t="shared" si="0"/>
         <v>3.13E-3</v>
       </c>
-      <c r="C14" s="17">
+      <c r="C14" s="12">
         <v>20</v>
       </c>
-      <c r="D14" s="17">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="17">
-        <v>1.0999999999999999E-2</v>
-      </c>
-      <c r="B15" s="17">
-        <v>3.1099999999999999E-3</v>
-      </c>
-      <c r="C15" s="17">
+      <c r="D14" s="12">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A15" s="12">
+        <v>8.0000000000000002E-3</v>
+      </c>
+      <c r="B15" s="8">
+        <f t="shared" si="0"/>
+        <v>3.0800000000000003E-3</v>
+      </c>
+      <c r="C15" s="12">
         <v>14</v>
       </c>
-      <c r="D15" s="17">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="17">
+      <c r="D15" s="12">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A16" s="12">
+        <v>6.0000000000000001E-3</v>
+      </c>
+      <c r="B16" s="8">
+        <f t="shared" si="0"/>
+        <v>3.0600000000000002E-3</v>
+      </c>
+      <c r="C16" s="12">
+        <v>10</v>
+      </c>
+      <c r="D16" s="12">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3272F67E-0749-4759-8ACF-9A1592264A89}">
+  <dimension ref="A1:D17"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A2" s="7">
+        <v>-0.18099999999999999</v>
+      </c>
+      <c r="B2" s="8">
+        <f t="shared" ref="B2:B16" si="0">ABS(A2*(1/100))+0.003</f>
+        <v>4.81E-3</v>
+      </c>
+      <c r="C2" s="7">
+        <v>80</v>
+      </c>
+      <c r="D2" s="8">
+        <f t="shared" ref="D2:D16" si="1">1/SQRT(12)</f>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A3" s="7">
+        <v>-0.124</v>
+      </c>
+      <c r="B3" s="8">
+        <f t="shared" si="0"/>
+        <v>4.2399999999999998E-3</v>
+      </c>
+      <c r="C3" s="7">
+        <v>74</v>
+      </c>
+      <c r="D3" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A4" s="7">
+        <v>-9.7000000000000003E-2</v>
+      </c>
+      <c r="B4" s="8">
+        <f t="shared" si="0"/>
+        <v>3.9700000000000004E-3</v>
+      </c>
+      <c r="C4" s="7">
+        <v>70</v>
+      </c>
+      <c r="D4" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A5" s="7">
+        <v>-7.6999999999999999E-2</v>
+      </c>
+      <c r="B5" s="8">
+        <f t="shared" si="0"/>
+        <v>3.7699999999999999E-3</v>
+      </c>
+      <c r="C5" s="7">
+        <v>64</v>
+      </c>
+      <c r="D5" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A6" s="9">
+        <v>-6.8000000000000005E-2</v>
+      </c>
+      <c r="B6" s="8">
+        <f t="shared" si="0"/>
+        <v>3.6800000000000001E-3</v>
+      </c>
+      <c r="C6" s="7">
+        <v>60</v>
+      </c>
+      <c r="D6" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A7" s="7">
+        <v>-4.9000000000000002E-2</v>
+      </c>
+      <c r="B7" s="8">
+        <f t="shared" si="0"/>
+        <v>3.49E-3</v>
+      </c>
+      <c r="C7" s="7">
+        <v>54</v>
+      </c>
+      <c r="D7" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A8" s="7">
+        <v>-4.3999999999999997E-2</v>
+      </c>
+      <c r="B8" s="8">
+        <f t="shared" si="0"/>
+        <v>3.4399999999999999E-3</v>
+      </c>
+      <c r="C8" s="7">
+        <v>50</v>
+      </c>
+      <c r="D8" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A9" s="7">
+        <v>-3.7999999999999999E-2</v>
+      </c>
+      <c r="B9" s="8">
+        <f t="shared" si="0"/>
+        <v>3.3800000000000002E-3</v>
+      </c>
+      <c r="C9" s="7">
+        <v>44</v>
+      </c>
+      <c r="D9" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A10" s="7">
+        <v>-3.3000000000000002E-2</v>
+      </c>
+      <c r="B10" s="8">
+        <f t="shared" si="0"/>
+        <v>3.3300000000000001E-3</v>
+      </c>
+      <c r="C10" s="7">
+        <v>40</v>
+      </c>
+      <c r="D10" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A11" s="7">
+        <v>-2.4E-2</v>
+      </c>
+      <c r="B11" s="8">
+        <f t="shared" si="0"/>
+        <v>3.2400000000000003E-3</v>
+      </c>
+      <c r="C11" s="7">
+        <v>34</v>
+      </c>
+      <c r="D11" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A12" s="7">
+        <v>-2.3E-2</v>
+      </c>
+      <c r="B12" s="8">
+        <f t="shared" si="0"/>
+        <v>3.2300000000000002E-3</v>
+      </c>
+      <c r="C12" s="7">
+        <v>30</v>
+      </c>
+      <c r="D12" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A13" s="7">
+        <v>-1.4999999999999999E-2</v>
+      </c>
+      <c r="B13" s="8">
+        <f t="shared" si="0"/>
+        <v>3.15E-3</v>
+      </c>
+      <c r="C13" s="7">
+        <v>24</v>
+      </c>
+      <c r="D13" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A14" s="9">
+        <v>-1.4E-2</v>
+      </c>
+      <c r="B14" s="8">
+        <f t="shared" si="0"/>
+        <v>3.14E-3</v>
+      </c>
+      <c r="C14" s="7">
+        <v>20</v>
+      </c>
+      <c r="D14" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A15" s="7">
+        <v>-8.9999999999999993E-3</v>
+      </c>
+      <c r="B15" s="8">
+        <f t="shared" si="0"/>
+        <v>3.0899999999999999E-3</v>
+      </c>
+      <c r="C15" s="7">
+        <v>14</v>
+      </c>
+      <c r="D15" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A16" s="7">
+        <v>-7.0000000000000001E-3</v>
+      </c>
+      <c r="B16" s="8">
+        <f t="shared" si="0"/>
+        <v>3.0700000000000002E-3</v>
+      </c>
+      <c r="C16" s="7">
+        <v>10</v>
+      </c>
+      <c r="D16" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="17" ht="15" thickTop="1"/>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89BC9873-1E51-46E1-A7DC-D38C19CF1588}">
+  <dimension ref="A1:D17"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData>
+    <row r="1" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A2" s="7">
+        <v>0.251</v>
+      </c>
+      <c r="B2" s="8">
+        <f t="shared" ref="B2:B16" si="0">ABS(A2*(1/100))+0.003</f>
+        <v>5.5100000000000001E-3</v>
+      </c>
+      <c r="C2" s="7">
+        <v>80</v>
+      </c>
+      <c r="D2" s="8">
+        <f t="shared" ref="D2:D16" si="1">1/SQRT(12)</f>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A3" s="7">
+        <v>0.14399999999999999</v>
+      </c>
+      <c r="B3" s="8">
+        <f t="shared" si="0"/>
+        <v>4.4399999999999995E-3</v>
+      </c>
+      <c r="C3" s="7">
+        <v>74</v>
+      </c>
+      <c r="D3" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A4" s="7">
+        <v>0.10299999999999999</v>
+      </c>
+      <c r="B4" s="8">
+        <f t="shared" si="0"/>
+        <v>4.0299999999999997E-3</v>
+      </c>
+      <c r="C4" s="7">
+        <v>70</v>
+      </c>
+      <c r="D4" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A5" s="7">
+        <v>7.6999999999999999E-2</v>
+      </c>
+      <c r="B5" s="8">
+        <f t="shared" si="0"/>
+        <v>3.7699999999999999E-3</v>
+      </c>
+      <c r="C5" s="7">
+        <v>64</v>
+      </c>
+      <c r="D5" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A6" s="9">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="B6" s="8">
+        <f t="shared" si="0"/>
+        <v>3.7000000000000002E-3</v>
+      </c>
+      <c r="C6" s="7">
+        <v>60</v>
+      </c>
+      <c r="D6" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A7" s="7">
+        <v>5.2999999999999999E-2</v>
+      </c>
+      <c r="B7" s="8">
+        <f t="shared" si="0"/>
+        <v>3.5300000000000002E-3</v>
+      </c>
+      <c r="C7" s="7">
+        <v>54</v>
+      </c>
+      <c r="D7" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A8" s="7">
+        <v>4.4999999999999998E-2</v>
+      </c>
+      <c r="B8" s="8">
+        <f t="shared" si="0"/>
+        <v>3.4499999999999999E-3</v>
+      </c>
+      <c r="C8" s="7">
+        <v>50</v>
+      </c>
+      <c r="D8" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A9" s="7">
+        <v>3.5999999999999997E-2</v>
+      </c>
+      <c r="B9" s="8">
+        <f t="shared" si="0"/>
+        <v>3.3600000000000001E-3</v>
+      </c>
+      <c r="C9" s="7">
+        <v>44</v>
+      </c>
+      <c r="D9" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A10" s="7">
+        <v>0.03</v>
+      </c>
+      <c r="B10" s="8">
+        <f t="shared" si="0"/>
+        <v>3.3E-3</v>
+      </c>
+      <c r="C10" s="7">
+        <v>40</v>
+      </c>
+      <c r="D10" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A11" s="7">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="B11" s="8">
+        <f t="shared" si="0"/>
+        <v>3.2500000000000003E-3</v>
+      </c>
+      <c r="C11" s="7">
+        <v>34</v>
+      </c>
+      <c r="D11" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A12" s="7">
+        <v>1.9E-2</v>
+      </c>
+      <c r="B12" s="8">
+        <f t="shared" si="0"/>
+        <v>3.1900000000000001E-3</v>
+      </c>
+      <c r="C12" s="7">
+        <v>30</v>
+      </c>
+      <c r="D12" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A13" s="7">
+        <v>1.6E-2</v>
+      </c>
+      <c r="B13" s="8">
+        <f t="shared" si="0"/>
+        <v>3.16E-3</v>
+      </c>
+      <c r="C13" s="7">
+        <v>24</v>
+      </c>
+      <c r="D13" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A14" s="7">
+        <v>1.2E-2</v>
+      </c>
+      <c r="B14" s="8">
+        <f t="shared" si="0"/>
+        <v>3.1199999999999999E-3</v>
+      </c>
+      <c r="C14" s="7">
+        <v>20</v>
+      </c>
+      <c r="D14" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A15" s="7">
         <v>8.0000000000000002E-3</v>
       </c>
-      <c r="B16" s="17">
-        <v>3.0799999999999998E-3</v>
-      </c>
-      <c r="C16" s="17">
+      <c r="B15" s="8">
+        <f t="shared" si="0"/>
+        <v>3.0800000000000003E-3</v>
+      </c>
+      <c r="C15" s="7">
+        <v>14</v>
+      </c>
+      <c r="D15" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="16.5" thickTop="1" thickBot="1">
+      <c r="A16" s="7">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="B16" s="8">
+        <f t="shared" si="0"/>
+        <v>3.0500000000000002E-3</v>
+      </c>
+      <c r="C16" s="7">
         <v>10</v>
       </c>
-      <c r="D16" s="17">
-        <v>0.28867513459999999</v>
-      </c>
-    </row>
+      <c r="D16" s="8">
+        <f t="shared" si="1"/>
+        <v>0.28867513459481292</v>
+      </c>
+    </row>
+    <row r="17" ht="15" thickTop="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>